<commit_message>
Leads: 2026-09-18 00:04 UTC (cycle 182)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -584,7 +584,6 @@
           <t>https://greentrucks.com/</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
           <t>info@greentrucks.com</t>
@@ -614,6 +613,238 @@
         </is>
       </c>
       <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Happy Plumbing</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>happyplumbing.net</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>https://happyplumbing.net/emergency-plumbing-mesa/</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Happy Plumbing</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>info@happyplumbing.net</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>(480) 528-9479</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Mesa AZ</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>100</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>emergency plumber Mesa AZ</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>All-Side Roofing &amp; Restoration LLC</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>allsideroof.com</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>https://allsideroof.com/roof-replacement-dayton-oh/</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Owner Owner</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>info@allsideroof.com</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>937-975-2363</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Dayton OH</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>90</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>roof replacement Dayton OH</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Rochester, MN Roofing Contractor | Ronningen Roofing</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>ronningenroofing.com</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>https://ronningenroofing.com/</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>eric@erroofing.com</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>(507) 281-8899</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Rochester MN</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>82</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>roofing contractor Rochester MN</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>24/7 Local Plumber in Mesa, AZ</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>oxplumbing.com</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>https://oxplumbing.com/emergency-plumbing</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>info@oxplumbingaz.com</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>(602) 905-3722</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Mesa AZ</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>80</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>emergency plumber Mesa AZ</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-18 00:06 UTC (cycle 183)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -759,7 +759,6 @@
           <t>https://ronningenroofing.com/</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>eric@erroofing.com</t>
@@ -815,7 +814,6 @@
           <t>https://oxplumbing.com/emergency-plumbing</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>info@oxplumbingaz.com</t>
@@ -845,6 +843,66 @@
         </is>
       </c>
       <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Water Heater Repair Olathe, KS | Garrison Plumbing</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>garrisonplumbing.com</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>https://www.garrisonplumbing.com/water-heater-repair</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>How Tankless</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>admin@garrisonservicesinc.com</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>(913) 768-1311</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Olathe KS</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>100</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>water heater repair Olathe KS</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-18 00:11 UTC (cycle 187)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -908,6 +908,182 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Plumbing Company Colorado</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>plumbingcompanycolorado.com</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>https://plumbingcompanycolorado.com/boulder/</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Gary Simmons</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>dispatch@plumbingcompanycolorado.com</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>303-567-7708</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Boulder CO</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>100</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>emergency plumber Boulder CO</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Canyon Plumbing &amp; Heating</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>canyonplumbers.com</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>https://canyonplumbers.com/</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>At Canyon</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>service@canyonplumbers.com</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>720-480-6228</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Boulder CO</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>100</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>emergency plumber Boulder CO</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>24 Hour Emergency Plumber in Boulder, CO</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>emergencyplumberboulder.com</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>https://emergencyplumberboulder.com/</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>admin@predictiveyield.com</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>303-218-4894</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Boulder CO</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>90</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>emergency plumber Boulder CO</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-18 00:17 UTC (cycle 191)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1049,7 +1049,6 @@
           <t>https://emergencyplumberboulder.com/</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
           <t>admin@predictiveyield.com</t>
@@ -1079,6 +1078,66 @@
         </is>
       </c>
       <c r="L11" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Greener Cleaner Heating &amp; Cooling HVAC LLC</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>greenercleanerheating.com</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>https://greenercleanerheating.com/federal-way-air-conditioning-repair/</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Federal Way</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>contact.greenercleanerheating@gmail.com</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>(253) 528-5482</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Federal Way WA</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>90</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>air conditioning repair Federal Way WA</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-18 00:19 UTC (cycle 192)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:L15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1143,6 +1143,186 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Bass Air Conditioning Co. - Fayetteville’s Trusted HVAC &amp; Plumbing Services Sinc</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>bass-air.com</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>https://bass-air.com/services/cooling/air-conditioning/</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Ed Leezer</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>support@bass-air.com</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>(910) 236-9210</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Fayetteville NC</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>90</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>AC installation Fayetteville NC</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Elk Grove Sewer &amp; Drain | Camera Inspection First</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>platinumpipesolutionsllc.com</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>https://www.platinumpipesolutionsllc.com/service-area/elk-grove/sewer-drain</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Platinum Pipe</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>platinumpipesolutions@gmail.com</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>(279) 209-1798</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Elk Grove CA</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>90</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>sewer repair Elk Grove CA</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Bringhurst Plumbing &amp; Heating</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>bringhurstplumbing.com</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>https://www.bringhurstplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Who We</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>info@bringhurstplumbing.com</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>(435) 673-6227</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>St George UT</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>88</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>plumber St George UT</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-18 00:22 UTC (cycle 194)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L15"/>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1323,6 +1323,66 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Top Rated Plumber in and around Bonita Springs</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>roccoswaterworks.com</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>https://roccoswaterworks.com/naples/</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Water Works</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>roccoswaterworks239@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>(239) 849-0809</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Naples FL</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>100</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>emergency plumber Naples FL</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-18 00:26 UTC (cycle 197)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L16"/>
+  <dimension ref="A1:L17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1383,6 +1383,66 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Residential Roofing Services</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>residentialroofingsc.com</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>https://www.residentialroofingsc.com/</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Residential Roofing</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>info@residentialroofingsc.com</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>(803) 629-4171</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Columbia SC</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>88</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>residential roofing company Columbia SC</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-18 00:32 UTC (cycle 201)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L17"/>
+  <dimension ref="A1:L18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1443,6 +1443,62 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>We Do Roofing Salt Lake City | High-quality Roofing Services</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>wedoroofingslc.com</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>https://wedoroofingslc.com/residential-roofing/</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>gabe@gkcconstruction.com</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>801-953-2877</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Salt Lake City UT</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>100</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>residential roofing company Salt Lake City UT</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-18 00:38 UTC (cycle 205)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L18"/>
+  <dimension ref="A1:L19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1464,7 +1464,6 @@
           <t>https://wedoroofingslc.com/residential-roofing/</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr">
         <is>
           <t>gabe@gkcconstruction.com</t>
@@ -1494,6 +1493,66 @@
         </is>
       </c>
       <c r="L18" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Aquashield Roofing Corporation</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>vbroof.com</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>https://aquashieldroof.com/virginia-beach/</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Roofers Located</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>jeff@vbroof.com</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>757-553-5191</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Norfolk VA</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>100</v>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>roof replacement Norfolk VA</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-18 12:53 UTC (cycle 3)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L19"/>
+  <dimension ref="A1:L20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1558,6 +1558,62 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>AZ Home Services Group - AC Repair &amp; Plumbing Services</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>azhomeservices.group</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>https://azhomeservices.group/service/repair-sewer/</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>info@azhomeservices.group</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>(602) 806-7212</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Tempe AZ</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>76</v>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>sewer repair Tempe AZ</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-18 12:54 UTC (cycle 4)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L20"/>
+  <dimension ref="A1:L21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1579,7 +1579,6 @@
           <t>https://azhomeservices.group/service/repair-sewer/</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
           <t>info@azhomeservices.group</t>
@@ -1609,6 +1608,66 @@
         </is>
       </c>
       <c r="L20" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Affordable Roofing Systems</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>affordableroofingflorida.com</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>https://www.affordableroofingflorida.com/affordable-roofing-services/roof-replacement/</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Winning Awards</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>info@affordableroofingflorida.com</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>(813) 542 8462</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Tampa FL</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
+        <v>90</v>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>roof replacement Tampa FL</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-18 12:57 UTC (cycle 6)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L21"/>
+  <dimension ref="A1:L22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1673,6 +1673,62 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Skelton's Heating, Cooling &amp; Plumbing</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>skeltonsair.com</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>https://skeltonsair.com/air-conditioning/ac-repair/</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>service@skeltonsair.com</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>(205) 289-3413</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Birmingham AL</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>100</v>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>air conditioning repair Birmingham AL</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-18 12:59 UTC (cycle 7)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L22"/>
+  <dimension ref="A1:L24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1694,7 +1694,6 @@
           <t>https://skeltonsair.com/air-conditioning/ac-repair/</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr">
         <is>
           <t>service@skeltonsair.com</t>
@@ -1724,6 +1723,126 @@
         </is>
       </c>
       <c r="L22" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Metal Roofing Installation in Rockford &amp; Machesney Park IL - Castle Contracting</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>castleexteriors.net</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>https://castleexteriors.net/metal-roof</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Brad Steele</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>info@castleexteriors.net</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>(877) 512-4207</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Rockford IL</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>90</v>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Rockford IL</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Roscoe Brown</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>roscoebrown.com</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>https://roscoebrown.com/</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Middle Tennessee</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>info@roscoebrown.com</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>(615) 203-3874</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Murfreesboro TN</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>90</v>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>HVAC contractor Murfreesboro TN</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-18 13:00 UTC (cycle 8)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L24"/>
+  <dimension ref="A1:L25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1848,6 +1848,66 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Roofing Contractor in Davenport, IA | Twin Bridge Roofing</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>roofqc.com</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>https://www.roofqc.com/davenport-iowa</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Twin Bridge</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>info@roofqc.com</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>(309) 948-4126</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Davenport IA</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>90</v>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>roofing contractor Davenport IA</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-18 13:02 UTC (cycle 9)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L25"/>
+  <dimension ref="A1:L26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1908,6 +1908,62 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Drain Cleaning | Columbia, MD | 410-933-8688</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>sunshine-plumbing.net</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>https://www.sunshine-plumbing.net/drain-cleaning/columbia-md</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>msopersr@callsunshine.plumbing</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>410-933-8688</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Columbia MD</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>100</v>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>drain cleaning service Columbia MD</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-18 13:05 UTC (cycle 11)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L26"/>
+  <dimension ref="A1:L27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1929,7 +1929,6 @@
           <t>https://www.sunshine-plumbing.net/drain-cleaning/columbia-md</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr">
         <is>
           <t>msopersr@callsunshine.plumbing</t>
@@ -1959,6 +1958,66 @@
         </is>
       </c>
       <c r="L26" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>OKC Roofing &amp; Contracting Group</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>okcroofingandcontracting.com</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>https://www.okcroofingandcontracting.com/residential-roofing/</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Oklahoma City</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>okcroofing.contracting@gmail.com</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>(405) 668-3996</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Edmond OK</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>100</v>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>residential roofing company Edmond OK</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-18 13:06 UTC (cycle 12)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L27"/>
+  <dimension ref="A1:L28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2023,6 +2023,66 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Guy Smith Heating, Cooling &amp; Plumbing</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>guysmithhomeservices.com</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>https://guysmithhomeservices.com/hvac-services/heating/heat-pump/</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Virginia Beach</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>admin@guysmith.net</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>(757) 913-9504</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Virginia Beach VA</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>100</v>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>heat pump installation Virginia Beach VA</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-18 13:08 UTC (cycle 13)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L28"/>
+  <dimension ref="A1:L30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2083,6 +2083,122 @@
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Pocatello Roofing &amp; Siding</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>metalmanconstruction.com</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>https://www.metalmanconstruction.com/pocatello-roofing-siding</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>office@metalmanconstruction.com</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>208-745-8440</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Pocatello ID</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
+        <v>86</v>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>roof replacement Pocatello ID</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Idaho Elite Roofing</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>idahoeliteroofing.com</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>https://idahoeliteroofing.com/</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Idaho Elite</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>idahoeliteroofing@gmail.com</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>(208) 223-2347</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Pocatello ID</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
+        <v>78</v>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>roof replacement Pocatello ID</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-18 13:11 UTC (cycle 15)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L30"/>
+  <dimension ref="A1:L31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2104,7 +2104,6 @@
           <t>https://www.metalmanconstruction.com/pocatello-roofing-siding</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
           <t>office@metalmanconstruction.com</t>
@@ -2194,6 +2193,66 @@
         </is>
       </c>
       <c r="L30" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Tempe AC Installation</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>alphasheatingandcooling.com</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>https://alphasheatingandcooling.com/tempe-ac-installation</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Tempe Town</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>joshua@nvmarketingco.com</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>(480) 709-5684</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Tempe AZ</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
+        <v>90</v>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>AC installation Tempe AZ</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-18 13:19 UTC (cycle 21)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L31"/>
+  <dimension ref="A1:L35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2258,6 +2258,238 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Believe Plumbing</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>believeplumbing.com</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>https://believeplumbing.com/drain-cleaning-services/st-petersburg/</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Believe Plumbing</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>believeplumbing@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>(813) 516-4486</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>St Petersburg FL</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
+        <v>90</v>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>drain cleaning service St Petersburg FL</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Douglas Roofing - Since 1985 | North Chesterfield, Richmond VA</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>douglasroofs.com</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>https://www.douglasroofs.com/locations/richmond</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>View Service</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>kyle@douglasroofs.com</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>(703) 255-9599</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Richmond VA</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
+        <v>88</v>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>roofing contractor Richmond VA</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Plumbing Pasadena</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>plumbing--pasadena.com</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>http://plumbing--pasadena.com/sewer-repair.html</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>service@plumbing--pasadena.com</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>281-826-2153</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Pasadena TX</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
+        <v>88</v>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>sewer repair Pasadena TX</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>TownVue</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>townvue.com</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>https://www.townvue.com/in/richmond-va/top/roofers</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Tad Rhodes</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>support@townvue.com</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Richmond VA</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
+        <v>74</v>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>roofing contractor Richmond VA</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-18 13:21 UTC (cycle 22)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L35"/>
+  <dimension ref="A1:L36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2399,7 +2399,6 @@
           <t>http://plumbing--pasadena.com/sewer-repair.html</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr"/>
       <c r="F34" t="inlineStr">
         <is>
           <t>service@plumbing--pasadena.com</t>
@@ -2465,7 +2464,6 @@
           <t>support@townvue.com</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr">
         <is>
           <t>Richmond VA</t>
@@ -2485,6 +2483,66 @@
         </is>
       </c>
       <c r="L35" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Roof Pros Arlington VA</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>roofprosarlingtonva.com</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>https://roofprosarlingtonva.com/</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Roof Pros</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>info@roofprosarlingtonva.com</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>(571) 605-1440</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Arlington VA</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
+        <v>90</v>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>roofer Arlington VA</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-18 13:25 UTC (cycle 25)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L36"/>
+  <dimension ref="A1:L37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2548,6 +2548,66 @@
         </is>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Professional Hvac Services | HVAC Contractor Provo</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>hvaccontractorprovo.com</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>https://hvaccontractorprovo.com/</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Testimonials What</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>info@hvaccontractorprovo.com</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>(855) 529-0128</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Provo UT</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
+        <v>90</v>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>HVAC contractor Provo UT</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-18 13:28 UTC (cycle 27)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L37"/>
+  <dimension ref="A1:L38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2608,6 +2608,66 @@
         </is>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Roof Maintenance | Rainbow Roof Maintenance | Honolulu, Pearl City &amp; Waipahu, HI</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>rainbowroof.com</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>https://www.rainbowroof.com/</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Why Choose</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>rrm@hawaiiantel.net</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>(808) 842-0488</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Honolulu HI</t>
+        </is>
+      </c>
+      <c r="I38" t="n">
+        <v>90</v>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>roof repair company Honolulu HI</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-18 13:31 UTC (cycle 29)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L38"/>
+  <dimension ref="A1:L41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2668,6 +2668,182 @@
         </is>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Davis Air-Tec</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>davisairtec.com</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>https://www.davisairtec.com/air-conditioning-installation-replacement-in-st-george-ut/</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>George Serving</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>davisairtec@gmail.com</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>435-635-4451</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>St George UT</t>
+        </is>
+      </c>
+      <c r="I39" t="n">
+        <v>90</v>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>AC installation St George UT</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Epsom Plumbing &amp; Heating</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>epsomplumbingandheating.com</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>https://epsomplumbingandheating.com/concord-nh-plumbing-company/</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>New Hampshire</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>epsomplumbingandheating@gmail.com</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>(603) 988-2853</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Concord NH</t>
+        </is>
+      </c>
+      <c r="I40" t="n">
+        <v>90</v>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>plumbing company Concord NH</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Air Rescue</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>airrescue.net</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>https://www.airrescue.net/ac-installation</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Washington County</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>office@airrescue.net</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr"/>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>St George UT</t>
+        </is>
+      </c>
+      <c r="I41" t="n">
+        <v>66</v>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>AC installation St George UT</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-18 13:36 UTC (cycle 32)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L41"/>
+  <dimension ref="A1:L42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2819,7 +2819,6 @@
           <t>office@airrescue.net</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr">
         <is>
           <t>St George UT</t>
@@ -2839,6 +2838,66 @@
         </is>
       </c>
       <c r="L41" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Military Plumbing</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>militaryplumbing.com</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>https://www.militaryplumbing.com/plumber-plano-tx</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Hunt County</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>service@militaryplumbing.com</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>972-635-7676</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Plano TX</t>
+        </is>
+      </c>
+      <c r="I42" t="n">
+        <v>100</v>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>plumber Plano TX</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-18 13:41 UTC (cycle 36)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L42"/>
+  <dimension ref="A1:L44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2903,6 +2903,122 @@
         </is>
       </c>
     </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Queens HVAC Services | Brooklyn Queens HVAC</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>brooklynqueenshvac.com</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>https://brooklynqueenshvac.com/ac-repair-queens-ny/</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr"/>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>brooklynqueenshvac@gmail.com</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>718-649-9000</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Queens NY</t>
+        </is>
+      </c>
+      <c r="I43" t="n">
+        <v>100</v>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>air conditioning repair Queens NY</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Air Conditioning Repair Staten Island, NY</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>bestheatingandairconditioning.com</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>https://www.bestheatingandairconditioning.com/</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Staten Island</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>bestts@aol.com</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>(718) 568-0573</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Staten Island NY</t>
+        </is>
+      </c>
+      <c r="I44" t="n">
+        <v>90</v>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>air conditioning repair Staten Island NY</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-18 13:52 UTC (cycle 43)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L44"/>
+  <dimension ref="A1:L45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2924,7 +2924,6 @@
           <t>https://brooklynqueenshvac.com/ac-repair-queens-ny/</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr"/>
       <c r="F43" t="inlineStr">
         <is>
           <t>brooklynqueenshvac@gmail.com</t>
@@ -3014,6 +3013,66 @@
         </is>
       </c>
       <c r="L44" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Elevated Roofing Solutions</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>elevatedroofingsolutions.org</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>https://elevatedroofingsolutions.org/roofing-company-sandy-springs-ga/</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Most Sandy</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>travis@elevatedroofingsolutions.org</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>(404) 626-3919</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Sandy Springs GA</t>
+        </is>
+      </c>
+      <c r="I45" t="n">
+        <v>90</v>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>residential roofing company Sandy Springs GA</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-18 14:02 UTC (cycle 50)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L45"/>
+  <dimension ref="A1:L47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3078,6 +3078,126 @@
         </is>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Heat Pump Installation Services | Pittsburgh, PA</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>zcwillishvac.com</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>https://www.zcwillishvac.com/heat-pump-installation</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Your Home</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>zcwillisheatingandcooling@gmail.com</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>(724) 747-7977</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Pittsburgh PA</t>
+        </is>
+      </c>
+      <c r="I46" t="n">
+        <v>100</v>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>heat pump installation Pittsburgh PA</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Parkis Air Care</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>parkisac.com</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>https://parkisac.com/heating-repairs/</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Jason Parkis</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>office@parkisac.com</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>(432) 570 0790</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Midland TX</t>
+        </is>
+      </c>
+      <c r="I47" t="n">
+        <v>88</v>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>furnace repair Midland TX</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-18 14:09 UTC (cycle 55)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L47"/>
+  <dimension ref="A1:L48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3198,6 +3198,66 @@
         </is>
       </c>
     </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Worcester HVAC Pros</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>worcesterhvacpros.com</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>https://worcesterhvacpros.com/</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Better Standard</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>ksvk18@gmail.com</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>(774) 436-6807</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Worcester MA</t>
+        </is>
+      </c>
+      <c r="I48" t="n">
+        <v>90</v>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>heating and cooling company Worcester MA</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-18 14:12 UTC (cycle 57)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L48"/>
+  <dimension ref="A1:L49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3258,6 +3258,66 @@
         </is>
       </c>
     </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Roofing Contractor Minneapolis MN</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>twsremodeling.com</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>https://twsremodeling.com/services/roofing/</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Roofing Contractors</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>info@twsremodeling.com</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>(612) 445-4352</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Minneapolis MN</t>
+        </is>
+      </c>
+      <c r="I49" t="n">
+        <v>100</v>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>roofing contractor Minneapolis MN</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-18 14:15 UTC (cycle 59)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L49"/>
+  <dimension ref="A1:L50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3318,6 +3318,66 @@
         </is>
       </c>
     </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Muetzel Heating and Cooling and Plumbing</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>muetzel.com</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>https://muetzel.com/</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Central Ohio</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>service@muetzel.com</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>(614) 299-7700</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Columbus OH</t>
+        </is>
+      </c>
+      <c r="I50" t="n">
+        <v>100</v>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>plumbing company Columbus OH</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-18 14:23 UTC (cycle 64)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L50"/>
+  <dimension ref="A1:L56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3378,6 +3378,358 @@
         </is>
       </c>
     </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Roof MD</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>roofmd.com</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>https://roofmd.com/roof-replacement-memphis/</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Standing Seam</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>gmancrocker@gmail.com</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>(901) 305-9136</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Memphis TN</t>
+        </is>
+      </c>
+      <c r="I51" t="n">
+        <v>100</v>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>roof replacement Memphis TN</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>No Limit Roofing</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>nolimitroofingmemphis.com</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>https://www.nolimitroofingmemphis.com/</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Assessment Homeowners</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>midsouthnolimitroofing@gmail.com</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>901-590-0058</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Memphis TN</t>
+        </is>
+      </c>
+      <c r="I52" t="n">
+        <v>100</v>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>roof replacement Memphis TN</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Chase Roof Inspections</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>chaseroofinspections.com</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>https://chaseroofinspections.com/roof-replacement-memphis-tn/</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Memphis Tri</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>john@chaseroofinspections.com</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>(901) 907-3666</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Memphis TN</t>
+        </is>
+      </c>
+      <c r="I53" t="n">
+        <v>100</v>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>roof replacement Memphis TN</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Home | Gonzalez Hvac Inc</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>gonzalezhvacinc.com</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>https://gonzalezhvacinc.com/</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr"/>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>mariogonzalez0879@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>818-438-0652</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Palmdale CA</t>
+        </is>
+      </c>
+      <c r="I54" t="n">
+        <v>96</v>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>HVAC contractor Palmdale CA</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>HVAC Installation &amp; Repair | Palmdale, CA | Garibay's A/C</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>garibaysheatingandair.com</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>https://www.garibaysheatingandair.com/</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr"/>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>garibaysac2023@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>(818) 836-2621</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Palmdale CA</t>
+        </is>
+      </c>
+      <c r="I55" t="n">
+        <v>90</v>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>HVAC contractor Palmdale CA</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Elite Roofing Solutions</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>ersmidsouth.com</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>https://www.ersmidsouth.com/roofreplacementmemphis</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Why Homeowners</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>info@ersmidsouth.com</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>(901) 435-6250</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Memphis TN</t>
+        </is>
+      </c>
+      <c r="I56" t="n">
+        <v>80</v>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>roof replacement Memphis TN</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-18 14:30 UTC (cycle 69)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L56"/>
+  <dimension ref="A1:L57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3579,7 +3579,6 @@
           <t>https://gonzalezhvacinc.com/</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr"/>
       <c r="F54" t="inlineStr">
         <is>
           <t>mariogonzalez0879@yahoo.com</t>
@@ -3635,7 +3634,6 @@
           <t>https://www.garibaysheatingandair.com/</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr"/>
       <c r="F55" t="inlineStr">
         <is>
           <t>garibaysac2023@yahoo.com</t>
@@ -3725,6 +3723,66 @@
         </is>
       </c>
       <c r="L56" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>On Point Roofing</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>onpointroofingdfw.com</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>https://onpointroofingdfw.com/service-areas/roofing-contractor-mckinney-tx/</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Page Schedule</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>austin@onpointroofingdfw.com</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>817-904-9423</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>McKinney TX</t>
+        </is>
+      </c>
+      <c r="I57" t="n">
+        <v>100</v>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>roof repair company McKinney TX</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-18 14:39 UTC (cycle 75)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L57"/>
+  <dimension ref="A1:L58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3788,6 +3788,62 @@
         </is>
       </c>
     </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Drain Openers</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>stldrainopeners.com</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>https://stldrainopeners.com/</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr"/>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>admin@stldrainopeners.com</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>(314) 996-9701</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>St Louis MO</t>
+        </is>
+      </c>
+      <c r="I58" t="n">
+        <v>90</v>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>drain cleaning service St Louis MO</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-18 14:46 UTC (cycle 80)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L58"/>
+  <dimension ref="A1:L59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3809,7 +3809,6 @@
           <t>https://stldrainopeners.com/</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr"/>
       <c r="F58" t="inlineStr">
         <is>
           <t>admin@stldrainopeners.com</t>
@@ -3839,6 +3838,66 @@
         </is>
       </c>
       <c r="L58" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>The BEST Roofing Company in Joliet - Commercial &amp; Residential</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>championroofing.com</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>https://championroofing.com/service-area/joliet</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Testimonials See</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>info@championroofing.com</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>(847) 673-7663</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>Joliet IL</t>
+        </is>
+      </c>
+      <c r="I59" t="n">
+        <v>90</v>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>residential roofing company Joliet IL</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-18 14:48 UTC (cycle 81)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L59"/>
+  <dimension ref="A1:L60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3903,6 +3903,66 @@
         </is>
       </c>
     </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Precision Bend Heating and Cooling</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>precisionbendheatingandcooling.com</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>http://precisionbendheatingandcooling.com/</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Sarah Jenkins</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>info@precisionbendheatingandcooling.com</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>(458) 292-2394</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>Bend OR</t>
+        </is>
+      </c>
+      <c r="I60" t="n">
+        <v>78</v>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>heating and cooling company Bend OR</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-18 14:49 UTC (cycle 82)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L60"/>
+  <dimension ref="A1:L61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3963,6 +3963,62 @@
         </is>
       </c>
     </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Cape Shore Plumbing</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>capeshoreplumbing.com</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>https://www.capeshoreplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr"/>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>info@capeshoreplumbing.com</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>(239) 677-9544</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>Cape Coral FL</t>
+        </is>
+      </c>
+      <c r="I61" t="n">
+        <v>90</v>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>plumber Cape Coral FL</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-18 14:52 UTC (cycle 84)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L61"/>
+  <dimension ref="A1:L64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3984,7 +3984,6 @@
           <t>https://www.capeshoreplumbing.com/</t>
         </is>
       </c>
-      <c r="E61" t="inlineStr"/>
       <c r="F61" t="inlineStr">
         <is>
           <t>info@capeshoreplumbing.com</t>
@@ -4014,6 +4013,182 @@
         </is>
       </c>
       <c r="L61" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Alpine Metal Roofing</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>alpineroofingak.com</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>https://www.alpineroofingak.com/</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr"/>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>john@alpineroofingak.com</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>(907) 671-6752</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>Anchorage AK</t>
+        </is>
+      </c>
+      <c r="I62" t="n">
+        <v>92</v>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Anchorage AK</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Northern Snow Removal</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>northernsnowremoval.co</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>https://northernsnowremoval.co/metal-roofing-anchorage</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Most Anchorage</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>northernsnowremoval382@gmail.com</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>(907) 317-7396</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>Anchorage AK</t>
+        </is>
+      </c>
+      <c r="I63" t="n">
+        <v>90</v>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Anchorage AK</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Anchorage, AK Metal Roofing Company</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>anchorage-ak.roofingrpgs.com</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>https://anchorage-ak.roofingrpgs.com/metal-roofing/</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Measurable Savings</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>info@roofingrpgs.com</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>(888) 766-0591</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>Anchorage AK</t>
+        </is>
+      </c>
+      <c r="I64" t="n">
+        <v>90</v>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Anchorage AK</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-18 14:58 UTC (cycle 88)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L64"/>
+  <dimension ref="A1:L65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4039,7 +4039,6 @@
           <t>https://www.alpineroofingak.com/</t>
         </is>
       </c>
-      <c r="E62" t="inlineStr"/>
       <c r="F62" t="inlineStr">
         <is>
           <t>john@alpineroofingak.com</t>
@@ -4189,6 +4188,66 @@
         </is>
       </c>
       <c r="L64" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Plumbing Emergency Pros</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>plumbingemergencypros.com</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>https://plumbingemergencypros.com/arkansas/jonesboro/</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Emergency Pros</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>service@plumbingemergencypros.com</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>877-373-9634</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>Jonesboro AR</t>
+        </is>
+      </c>
+      <c r="I65" t="n">
+        <v>90</v>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>emergency plumber Jonesboro AR</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-18 15:10 UTC (cycle 96)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L65"/>
+  <dimension ref="A1:L66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4253,6 +4253,62 @@
         </is>
       </c>
     </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Island Comfort</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>islandcomfort.com</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>https://islandcomfort.com/</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr"/>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>vfetty@islandcomfort.com</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>(808) 562-3971</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>Honolulu HI</t>
+        </is>
+      </c>
+      <c r="I66" t="n">
+        <v>98</v>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>heating and cooling company Honolulu HI</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-18 15:13 UTC (cycle 98)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L66"/>
+  <dimension ref="A1:L67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4274,7 +4274,6 @@
           <t>https://islandcomfort.com/</t>
         </is>
       </c>
-      <c r="E66" t="inlineStr"/>
       <c r="F66" t="inlineStr">
         <is>
           <t>vfetty@islandcomfort.com</t>
@@ -4304,6 +4303,66 @@
         </is>
       </c>
       <c r="L66" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Drain Cleaning in Port St Lucie | Florida Plumbing Services</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>callfloridaplumber.com</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>https://callfloridaplumber.com/locations/port-st-lucie/drain-cleaning</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Port St</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>hello@callfloridaplumber.com</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>833-830-0028</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>Port St Lucie FL</t>
+        </is>
+      </c>
+      <c r="I67" t="n">
+        <v>90</v>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>drain cleaning service Port St Lucie FL</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-18 15:17 UTC (cycle 101)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L67"/>
+  <dimension ref="A1:L68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4368,6 +4368,62 @@
         </is>
       </c>
     </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Apex Plumbing Repair</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>apexplumbingla.com</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>https://apexplumbingla.com/services/drain-cleaning-2/</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr"/>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>apexplumbingrepair@gmail.com</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>(337) 570-2794</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>Lafayette LA</t>
+        </is>
+      </c>
+      <c r="I68" t="n">
+        <v>90</v>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>drain cleaning service Lafayette LA</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-18 15:20 UTC (cycle 103)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L68"/>
+  <dimension ref="A1:L69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4389,7 +4389,6 @@
           <t>https://apexplumbingla.com/services/drain-cleaning-2/</t>
         </is>
       </c>
-      <c r="E68" t="inlineStr"/>
       <c r="F68" t="inlineStr">
         <is>
           <t>apexplumbingrepair@gmail.com</t>
@@ -4419,6 +4418,62 @@
         </is>
       </c>
       <c r="L68" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>All Star Plumbing</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>allstarplumbingfresno.com</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>https://allstarplumbingfresno.com/</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr"/>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>info@allstarplumbingfresno.com</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>(559) 445-9999</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>Fresno CA</t>
+        </is>
+      </c>
+      <c r="I69" t="n">
+        <v>100</v>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>sewer repair Fresno CA</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-18 15:30 UTC (cycle 110)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L69"/>
+  <dimension ref="A1:L70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4444,7 +4444,6 @@
           <t>https://allstarplumbingfresno.com/</t>
         </is>
       </c>
-      <c r="E69" t="inlineStr"/>
       <c r="F69" t="inlineStr">
         <is>
           <t>info@allstarplumbingfresno.com</t>
@@ -4474,6 +4473,66 @@
         </is>
       </c>
       <c r="L69" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Plumbing Repairs | Youngstown, OH</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>mahoningvalleyplumbinghtg.com</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>https://mahoningvalleyplumbinghtg.com/</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Mahoning Valley</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>mvph4663@icloud.com</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>(330) 746-4663</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>Youngstown OH</t>
+        </is>
+      </c>
+      <c r="I70" t="n">
+        <v>90</v>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>plumbing company Youngstown OH</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-18 15:45 UTC (cycle 120)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L70"/>
+  <dimension ref="A1:L71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4538,6 +4538,66 @@
         </is>
       </c>
     </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>HD Roofing and Repairs</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>hdroofingandrepairs.com</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>https://hdroofingandrepairs.com/austin/</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Central Texas</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>contact@hdroofingandrepairs.com</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>(512) 458-6800</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>Austin TX</t>
+        </is>
+      </c>
+      <c r="I71" t="n">
+        <v>90</v>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>residential roofing company Austin TX</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-18 15:46 UTC (cycle 121)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L71"/>
+  <dimension ref="A1:L72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4598,6 +4598,66 @@
         </is>
       </c>
     </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Rapid Sewer Cleaners</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>rapidsewerandsepticcleaners.com</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>https://rapidsewerandsepticcleaners.com/</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Services We</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>rapidswr@aol.com</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>(718) 720-5222</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>Staten Island NY</t>
+        </is>
+      </c>
+      <c r="I72" t="n">
+        <v>90</v>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>drain cleaning service Staten Island NY</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-18 15:49 UTC (cycle 123)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L72"/>
+  <dimension ref="A1:L73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4658,6 +4658,62 @@
         </is>
       </c>
     </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>G&amp;T Plumbing &amp; Mechanical</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>gandtplumbing.com</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>https://gandtplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr"/>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>josh@gandtplumbing.com</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>(406) 256-6016</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>Billings MT</t>
+        </is>
+      </c>
+      <c r="I73" t="n">
+        <v>80</v>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>plumbing company Billings MT</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-18 15:54 UTC (cycle 126)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L73"/>
+  <dimension ref="A1:L75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4679,7 +4679,6 @@
           <t>https://gandtplumbing.com/</t>
         </is>
       </c>
-      <c r="E73" t="inlineStr"/>
       <c r="F73" t="inlineStr">
         <is>
           <t>josh@gandtplumbing.com</t>
@@ -4709,6 +4708,126 @@
         </is>
       </c>
       <c r="L73" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>HVAC Repair in Lawton, OK | Furnace &amp; AC</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>quickhomeservices.org</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>https://www.quickhomeservices.org/hvac-repair-lawton-ok/</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Requests Made</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>help@quickhomeservices.org</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>(702) 745-8238</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>Lawton OK</t>
+        </is>
+      </c>
+      <c r="I74" t="n">
+        <v>90</v>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>furnace repair Lawton OK</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>ATM Roofing Solutions LLC</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>atmroofingsolutions.com</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>https://www.atmroofingsolutions.com/service-areas/san-marcos</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Services Ready</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>info@atmroofingsolutions.com</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>(737)-237-8060</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>San Marcos TX</t>
+        </is>
+      </c>
+      <c r="I75" t="n">
+        <v>90</v>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>roof replacement San Marcos TX</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-18 16:04 UTC (cycle 133)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L75"/>
+  <dimension ref="A1:L76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4833,6 +4833,66 @@
         </is>
       </c>
     </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>premierexteriorscr.com</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>premierexteriorscr.com</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>https://premierexteriorscr.com/roofing/</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Cedar Rapids</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>info@premierexteriorscr.com</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>(319) 671-6753</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>Cedar Rapids IA</t>
+        </is>
+      </c>
+      <c r="I76" t="n">
+        <v>100</v>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>roof replacement Cedar Rapids IA</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-18 16:07 UTC (cycle 135)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L76"/>
+  <dimension ref="A1:L78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4893,6 +4893,126 @@
         </is>
       </c>
     </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>2G exteriors</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>2gexteriors.com</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>https://2gexteriors.com/residential-roofing</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Stream Oak</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>info@2ghomesolutions.com</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>312-765-9500</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>Elgin IL</t>
+        </is>
+      </c>
+      <c r="I77" t="n">
+        <v>100</v>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>residential roofing company Elgin IL</t>
+        </is>
+      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>2G exteriors</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>2ghomesolutions.com</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>https://2ghomesolutions.com/residential-roofing</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Stream Oak</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>info@2ghomesolutions.com</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>312-765-9500</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>Elgin IL</t>
+        </is>
+      </c>
+      <c r="I78" t="n">
+        <v>100</v>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>residential roofing company Elgin IL</t>
+        </is>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-18 16:10 UTC (cycle 137)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L78"/>
+  <dimension ref="A1:L79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5013,6 +5013,62 @@
         </is>
       </c>
     </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Domco Plumbing</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>domcoplumbing.com</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>https://www.domcoplumbing.com/plumbing-repairs/sewer-repair/</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr"/>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>info@sfvalleyplumbing.com</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>916.353.0203</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>Sacramento CA</t>
+        </is>
+      </c>
+      <c r="I79" t="n">
+        <v>90</v>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>sewer repair Sacramento CA</t>
+        </is>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-18 16:33 UTC (cycle 153)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L79"/>
+  <dimension ref="A1:L80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5034,7 +5034,6 @@
           <t>https://www.domcoplumbing.com/plumbing-repairs/sewer-repair/</t>
         </is>
       </c>
-      <c r="E79" t="inlineStr"/>
       <c r="F79" t="inlineStr">
         <is>
           <t>info@sfvalleyplumbing.com</t>
@@ -5064,6 +5063,62 @@
         </is>
       </c>
       <c r="L79" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Burnett's Plumbing</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>burnettsplumbing.com</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>https://burnettsplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr"/>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>burnettsplumbing@outlook.com</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>(602) 472-1007</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>Surprise AZ</t>
+        </is>
+      </c>
+      <c r="I80" t="n">
+        <v>84</v>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>plumbing company Surprise AZ</t>
+        </is>
+      </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L80" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-18 16:34 UTC (cycle 154)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L80"/>
+  <dimension ref="A1:L81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5089,7 +5089,6 @@
           <t>https://burnettsplumbing.com/</t>
         </is>
       </c>
-      <c r="E80" t="inlineStr"/>
       <c r="F80" t="inlineStr">
         <is>
           <t>burnettsplumbing@outlook.com</t>
@@ -5119,6 +5118,66 @@
         </is>
       </c>
       <c r="L80" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Armory Plumbing Inc</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>armoryplumbinginc.com</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>https://armoryplumbinginc.com/</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Armory Plumbing</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>office@armoryplumbinginc.com</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>(978) 815-0895</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>Lowell MA</t>
+        </is>
+      </c>
+      <c r="I81" t="n">
+        <v>90</v>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>plumbing company Lowell MA</t>
+        </is>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L81" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-18 16:37 UTC (cycle 156)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L81"/>
+  <dimension ref="A1:L82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5183,6 +5183,62 @@
         </is>
       </c>
     </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Big Dawg Plumbing</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>bigdawgplumbingid.com</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>https://bigdawgplumbingid.com/drain-cleaning-boise-id/</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr"/>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>bigdawgplumbing1@gmail.com</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>986-777-1365</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>Boise ID</t>
+        </is>
+      </c>
+      <c r="I82" t="n">
+        <v>100</v>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>drain cleaning service Boise ID</t>
+        </is>
+      </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-18 16:39 UTC (cycle 157)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L82"/>
+  <dimension ref="A1:L83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5204,7 +5204,6 @@
           <t>https://bigdawgplumbingid.com/drain-cleaning-boise-id/</t>
         </is>
       </c>
-      <c r="E82" t="inlineStr"/>
       <c r="F82" t="inlineStr">
         <is>
           <t>bigdawgplumbing1@gmail.com</t>
@@ -5234,6 +5233,66 @@
         </is>
       </c>
       <c r="L82" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>California Green Roofing</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>californiagreenroofingremodeling.com</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>https://californiagreenroofingremodeling.com/roofing-long-beach-ca/</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Privacy Policy</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>cagreenroofing@gmail.com</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>747-298-6407</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>Long Beach CA</t>
+        </is>
+      </c>
+      <c r="I83" t="n">
+        <v>100</v>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Long Beach CA</t>
+        </is>
+      </c>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L83" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-18 16:44 UTC (cycle 161)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L83"/>
+  <dimension ref="A1:L85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5298,6 +5298,123 @@
         </is>
       </c>
     </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Vincent
+Plumbing</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>vincentplumbing.com</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>https://www.vincentplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr"/>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>amy@vincentplumbing.com</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>(262) 347-3322</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>Waukesha WI</t>
+        </is>
+      </c>
+      <c r="I84" t="n">
+        <v>100</v>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>plumber Waukesha WI</t>
+        </is>
+      </c>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Legacy Construction</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>legacyconstructionmn.com</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>https://legacyconstructionmn.com/service-areas/woodbury-mn-roofers/</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Installation We</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>info@legacyconstructionmn.com</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>(952) 303-4080</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>Woodbury MN</t>
+        </is>
+      </c>
+      <c r="I85" t="n">
+        <v>90</v>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>residential roofing company Woodbury MN</t>
+        </is>
+      </c>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L85" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-18 16:47 UTC (cycle 163)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L85"/>
+  <dimension ref="A1:L87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5320,7 +5320,6 @@
           <t>https://www.vincentplumbing.com/</t>
         </is>
       </c>
-      <c r="E84" t="inlineStr"/>
       <c r="F84" t="inlineStr">
         <is>
           <t>amy@vincentplumbing.com</t>
@@ -5410,6 +5409,122 @@
         </is>
       </c>
       <c r="L85" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Stones River Roofing</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>stonesriverroofing.com</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>https://stonesriverroofing.com/</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Middle Tennessee</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>office@stonesriverroofing.com</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>615-200-7753</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>Murfreesboro TN</t>
+        </is>
+      </c>
+      <c r="I86" t="n">
+        <v>100</v>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>residential roofing company Murfreesboro TN</t>
+        </is>
+      </c>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Southern Style Roof &amp; Home Exterior | Siding | Murfreesboro, TN</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>southernstyleroofexterior.com</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>https://www.southernstyleroofexterior.com/</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr"/>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>southernstyle615@gmail.com</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>(615) 307-9792</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>Murfreesboro TN</t>
+        </is>
+      </c>
+      <c r="I87" t="n">
+        <v>84</v>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>residential roofing company Murfreesboro TN</t>
+        </is>
+      </c>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L87" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-18 16:50 UTC (cycle 165)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L87"/>
+  <dimension ref="A1:L88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5495,7 +5495,6 @@
           <t>https://www.southernstyleroofexterior.com/</t>
         </is>
       </c>
-      <c r="E87" t="inlineStr"/>
       <c r="F87" t="inlineStr">
         <is>
           <t>southernstyle615@gmail.com</t>
@@ -5525,6 +5524,62 @@
         </is>
       </c>
       <c r="L87" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>All Pro Plumbing Heating and Air</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>allproplumbingheatingandair.com</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>https://allproplumbingheatingandair.com/services/furnace-repair/</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr"/>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>info@allproplumbingheatingandair.com</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>(661) 863-9242</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>Bakersfield CA</t>
+        </is>
+      </c>
+      <c r="I88" t="n">
+        <v>90</v>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>furnace repair Bakersfield CA</t>
+        </is>
+      </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L88" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-18 16:59 UTC (cycle 171)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L88"/>
+  <dimension ref="A1:L89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5550,7 +5550,6 @@
           <t>https://allproplumbingheatingandair.com/services/furnace-repair/</t>
         </is>
       </c>
-      <c r="E88" t="inlineStr"/>
       <c r="F88" t="inlineStr">
         <is>
           <t>info@allproplumbingheatingandair.com</t>
@@ -5580,6 +5579,66 @@
         </is>
       </c>
       <c r="L88" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>E.W. Tompkins Plumbing Heating Cooling</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>ewtompkins.com</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>https://www.ewtompkins.com/</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Heating Cooling</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>info@ewtompkins.com</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>(518) 462-6577</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>Albany NY</t>
+        </is>
+      </c>
+      <c r="I89" t="n">
+        <v>100</v>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>plumbing company Albany NY</t>
+        </is>
+      </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L89" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-18 17:09 UTC (cycle 178)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L89"/>
+  <dimension ref="A1:L90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5644,6 +5644,66 @@
         </is>
       </c>
     </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Signature Exteriors - A St. Charles and St. Louis Roofing Contractor</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>saintcharlesroofing.com</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>https://saintcharlesroofing.com/</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Jeramie Beechler</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>info@sigext.com</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>(314) 827-5376</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>St Charles MO</t>
+        </is>
+      </c>
+      <c r="I90" t="n">
+        <v>90</v>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>roofer St Charles MO</t>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-18 17:13 UTC (cycle 181)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L90"/>
+  <dimension ref="A1:L91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5704,6 +5704,62 @@
         </is>
       </c>
     </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Roof Repair | Erie, PA | Rash Roofing &amp; Siding</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>rashroofingandsiding.com</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>https://www.rashroofingandsiding.com/roof-repair</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr"/>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>rashroofing@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>(814) 403-0471</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>Erie PA</t>
+        </is>
+      </c>
+      <c r="I91" t="n">
+        <v>100</v>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>roof repair company Erie PA</t>
+        </is>
+      </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-18 17:15 UTC (cycle 182)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L91"/>
+  <dimension ref="A1:L95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5725,7 +5725,6 @@
           <t>https://www.rashroofingandsiding.com/roof-repair</t>
         </is>
       </c>
-      <c r="E91" t="inlineStr"/>
       <c r="F91" t="inlineStr">
         <is>
           <t>rashroofing@yahoo.com</t>
@@ -5755,6 +5754,238 @@
         </is>
       </c>
       <c r="L91" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Meyer Heating &amp; Air</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>meyerhvacmn.com</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>https://www.meyerhvacmn.com/bloomington/</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Meyer Heating</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>contact@meyerhvacmn.com</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>952-800-6768</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>Bloomington MN</t>
+        </is>
+      </c>
+      <c r="I92" t="n">
+        <v>98</v>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>air conditioning repair Bloomington MN</t>
+        </is>
+      </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Super Heat, Air, and Plumbing</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>superheatandair.com</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>https://superheatandair.com/hvac-services/heat-pump-installation/</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr"/>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>info@superheatandair.com</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>(813) 279-8213</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>Tampa FL</t>
+        </is>
+      </c>
+      <c r="I93" t="n">
+        <v>90</v>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>heat pump installation Tampa FL</t>
+        </is>
+      </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Blue Peak Air Conditioning, LLC</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>bluepeak-ac.com</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>https://www.bluepeak-ac.com/heat-pump-installation</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr"/>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>info@bluepeakairconditioning.com</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>(813) 572-2653</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>Tampa FL</t>
+        </is>
+      </c>
+      <c r="I94" t="n">
+        <v>90</v>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>heat pump installation Tampa FL</t>
+        </is>
+      </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Fisher Of Men HVAC and Construction LLC</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>fomhvacandconstruction.com</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>https://www.fomhvacandconstruction.com/</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Fisher Of</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>fomhvacandconstruction@gmail.com</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>(541) 517-9552</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>Eugene OR</t>
+        </is>
+      </c>
+      <c r="I95" t="n">
+        <v>80</v>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>HVAC contractor Eugene OR</t>
+        </is>
+      </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L95" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-18 17:16 UTC (cycle 183)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L95"/>
+  <dimension ref="A1:L96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5840,7 +5840,6 @@
           <t>https://superheatandair.com/hvac-services/heat-pump-installation/</t>
         </is>
       </c>
-      <c r="E93" t="inlineStr"/>
       <c r="F93" t="inlineStr">
         <is>
           <t>info@superheatandair.com</t>
@@ -5896,7 +5895,6 @@
           <t>https://www.bluepeak-ac.com/heat-pump-installation</t>
         </is>
       </c>
-      <c r="E94" t="inlineStr"/>
       <c r="F94" t="inlineStr">
         <is>
           <t>info@bluepeakairconditioning.com</t>
@@ -5986,6 +5984,66 @@
         </is>
       </c>
       <c r="L95" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Duty Calls Plumbing and Rooter</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>dutycallspr.com</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>https://dutycallspr.com/services/sewer-line-repair-and-replacement/</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Sewer Line</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>office@dutycallspr.com</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>(816) 945-2131</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>Independence MO</t>
+        </is>
+      </c>
+      <c r="I96" t="n">
+        <v>100</v>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>sewer repair Independence MO</t>
+        </is>
+      </c>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L96" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-18 17:18 UTC (cycle 184)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L96"/>
+  <dimension ref="A1:L97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6049,6 +6049,66 @@
         </is>
       </c>
     </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Pacific Appliance Solutions</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>pacificappliancesolutions.com</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>https://pacificappliancesolutions.com/hvac-repair-hillsboro-or/</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>Repair Service</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>support@pacificappliancesolutions.com</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>(360) 518-0254</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>Hillsboro OR</t>
+        </is>
+      </c>
+      <c r="I97" t="n">
+        <v>100</v>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>furnace repair Hillsboro OR</t>
+        </is>
+      </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L97" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-18 17:27 UTC (cycle 190)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L97"/>
+  <dimension ref="A1:L98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6109,6 +6109,66 @@
         </is>
       </c>
     </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Twisted Air</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>twistedairlaredo.com</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>https://www.twistedairlaredo.com/services/heating.html</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Owner Ignacio</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>nach1750@live.com</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>(956) 646-7957</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>Laredo TX</t>
+        </is>
+      </c>
+      <c r="I98" t="n">
+        <v>90</v>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>furnace repair Laredo TX</t>
+        </is>
+      </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-18 17:30 UTC (cycle 192)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L98"/>
+  <dimension ref="A1:L99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6169,6 +6169,66 @@
         </is>
       </c>
     </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Forge Roofing &amp; Exteriors</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>forgeroofingco.com</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>https://www.forgeroofingco.com/</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Fort Wayne</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>example@mysite.com</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>(260-255-4561</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>Fort Wayne IN</t>
+        </is>
+      </c>
+      <c r="I99" t="n">
+        <v>94</v>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>roofing contractor Fort Wayne IN</t>
+        </is>
+      </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-18 17:31 UTC (cycle 193)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L99"/>
+  <dimension ref="A1:L101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6229,6 +6229,126 @@
         </is>
       </c>
     </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>HVAC Contractor Thornton, CO | Savage Heating and Air</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>savageheatingnair.com</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>https://www.savageheatingnair.com/</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Why Most</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>savageheatingnair@gmail.com</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>(720) 242-5937</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>Thornton CO</t>
+        </is>
+      </c>
+      <c r="I100" t="n">
+        <v>100</v>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>HVAC contractor Thornton CO</t>
+        </is>
+      </c>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L100" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Perfect Time Builders - The Best Roofing and Exterior Company in Lincoln NE</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>perfecttimebuilders.com</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>https://perfecttimebuilders.com/residential-roofing-lincoln-ne/</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Roofing Specialists</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>info@perfecttimebuilders.com</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>(402) 326-9609</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>Lincoln NE</t>
+        </is>
+      </c>
+      <c r="I101" t="n">
+        <v>90</v>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>residential roofing company Lincoln NE</t>
+        </is>
+      </c>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L101" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-18 17:37 UTC (cycle 197)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L101"/>
+  <dimension ref="A1:L104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6349,6 +6349,186 @@
         </is>
       </c>
     </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Kabran Air Conditioning &amp; Heating</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>kabran.com</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>https://kabran.com/palm-bay-fl/</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>Kabran Air</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>kabranair@kabran.com</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>321-380-1601</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>Palm Bay FL</t>
+        </is>
+      </c>
+      <c r="I102" t="n">
+        <v>90</v>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>heating and cooling company Palm Bay FL</t>
+        </is>
+      </c>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L102" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Summit Construction</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>summitconstructionla.com</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>https://summitconstructionla.com/roofing-contractor-metairie/</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>Serving Southeast</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>info@summitconstructionla.com</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>504-418-1329</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>Metairie LA</t>
+        </is>
+      </c>
+      <c r="I103" t="n">
+        <v>90</v>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>roofing contractor Metairie LA</t>
+        </is>
+      </c>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L103" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Heating Services | Peoria, IL | Griffin HVAC</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>griffinheatingcooling.com</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>https://www.griffinheatingcooling.com/</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>Jane Ingersoll</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>douggriffinheatcool@gmail.com</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>309-676-0808</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>Peoria IL</t>
+        </is>
+      </c>
+      <c r="I104" t="n">
+        <v>88</v>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>heating and cooling company Peoria IL</t>
+        </is>
+      </c>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L104" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-18 17:40 UTC (cycle 199)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L104"/>
+  <dimension ref="A1:L106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6529,6 +6529,122 @@
         </is>
       </c>
     </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Emergency Plumbing in Roanoke, VA | Roanoke Plumbing Pros | (540) 302-5580</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>roanokevaplumbing.com</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>https://roanokevaplumbing.com/emergency-plumber</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>Roanoke Valley</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>support@roanokevaplumbing.com</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>(540) 302-5580</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>Roanoke VA</t>
+        </is>
+      </c>
+      <c r="I105" t="n">
+        <v>100</v>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>emergency plumber Roanoke VA</t>
+        </is>
+      </c>
+      <c r="K105" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L105" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>James Buck Plumbing &amp; Heating Inc | Plumber | Roanoke, VA</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>jamesbuckplumbingandheating.com</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>https://www.jamesbuckplumbingandheating.com/</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr"/>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>james@jbph.roacoxmail.com</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>540-774-7729</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>Roanoke VA</t>
+        </is>
+      </c>
+      <c r="I106" t="n">
+        <v>88</v>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>emergency plumber Roanoke VA</t>
+        </is>
+      </c>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L106" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-18 17:46 UTC (cycle 203)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L106"/>
+  <dimension ref="A1:L107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6610,7 +6610,6 @@
           <t>https://www.jamesbuckplumbingandheating.com/</t>
         </is>
       </c>
-      <c r="E106" t="inlineStr"/>
       <c r="F106" t="inlineStr">
         <is>
           <t>james@jbph.roacoxmail.com</t>
@@ -6640,6 +6639,66 @@
         </is>
       </c>
       <c r="L106" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Emergency Plumber | Yonkers, NY | Plumbing &amp; Heating By Woody</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>plumbingandheatingbywoody.com</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>https://www.plumbingandheatingbywoody.com/emergency-plumber/yonkers-ny</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Button Button</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>example@gmail.com</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>201-387-1368</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>Yonkers NY</t>
+        </is>
+      </c>
+      <c r="I107" t="n">
+        <v>100</v>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>emergency plumber Yonkers NY</t>
+        </is>
+      </c>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L107" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-18 18:58 UTC (cycle 2)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L107"/>
+  <dimension ref="A1:L108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6704,6 +6704,66 @@
         </is>
       </c>
     </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Emergency Plumber in Concord, NC</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>macawplumbing.com</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>https://www.macawplumbing.com/concord-nc-plumber/emergency-plumber</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>Jonathan Johns</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>contact@macawplumbing.com</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>(704) 798-2659</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>Concord NC</t>
+        </is>
+      </c>
+      <c r="I108" t="n">
+        <v>90</v>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>emergency plumber Concord NC</t>
+        </is>
+      </c>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L108" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-18 19:02 UTC (cycle 5)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L108"/>
+  <dimension ref="A1:L109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6764,6 +6764,66 @@
         </is>
       </c>
     </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Heat Pump Services in Appleton, WI | Conradt Quality Air</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>conradtqualityair.com</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>https://conradtqualityair.com/services/heat-pump-services</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Conradt Quality</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>conradtqualityair@gmail.com</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>(920) 636-8701</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>Appleton WI</t>
+        </is>
+      </c>
+      <c r="I109" t="n">
+        <v>90</v>
+      </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>heat pump installation Appleton WI</t>
+        </is>
+      </c>
+      <c r="K109" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L109" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-18 19:04 UTC (cycle 6)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L109"/>
+  <dimension ref="A1:L110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6824,6 +6824,62 @@
         </is>
       </c>
     </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Desert Diamond Air</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>desertdiamondhvac.com</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>https://desertdiamondhvac.com/</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr"/>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>noreply@desertdiamondhvac.com</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>602-362-4599</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>Phoenix AZ</t>
+        </is>
+      </c>
+      <c r="I110" t="n">
+        <v>90</v>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>air conditioning repair Phoenix AZ</t>
+        </is>
+      </c>
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L110" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-18 19:05 UTC (cycle 7)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L110"/>
+  <dimension ref="A1:L111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6845,7 +6845,6 @@
           <t>https://desertdiamondhvac.com/</t>
         </is>
       </c>
-      <c r="E110" t="inlineStr"/>
       <c r="F110" t="inlineStr">
         <is>
           <t>noreply@desertdiamondhvac.com</t>
@@ -6875,6 +6874,66 @@
         </is>
       </c>
       <c r="L110" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Ideal Roofing Inc.</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>idealroofinginc.com</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>https://idealroofinginc.com/</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Roofing Experts</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>info@idealroofinginc.com</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>(812) 666-0385</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>Evansville IN</t>
+        </is>
+      </c>
+      <c r="I111" t="n">
+        <v>100</v>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>roofing contractor Evansville IN</t>
+        </is>
+      </c>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L111" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-18 19:07 UTC (cycle 8)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L111"/>
+  <dimension ref="A1:L117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6939,6 +6939,362 @@
         </is>
       </c>
     </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Harbor Roofing and Siding</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>harborroofingandsiding.com</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>https://harborroofingandsiding.com/metal-roofing-in-wilmington-nc/</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>New Hanover</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>office@harborcompanies.org</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>(910) 262-5508</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>Wilmington NC</t>
+        </is>
+      </c>
+      <c r="I112" t="n">
+        <v>100</v>
+      </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Wilmington NC</t>
+        </is>
+      </c>
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L112" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Wilmington NC Metal Roofing</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>wilmingtonncmetalroofing.com</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>https://www.wilmingtonncmetalroofing.com/</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>Wilmingon Metal</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>info@gatormetalroofing.com</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>866-257-3619</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>Wilmington NC</t>
+        </is>
+      </c>
+      <c r="I113" t="n">
+        <v>96</v>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Wilmington NC</t>
+        </is>
+      </c>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L113" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Wilmington Roofing</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>wilmingtonroofingllc.com</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>https://wilmingtonroofingllc.com/metal-roofing/</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>Homeowners Across</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>cb@digitalrainmaker.co.uk</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>910-548-7922</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>Wilmington NC</t>
+        </is>
+      </c>
+      <c r="I114" t="n">
+        <v>90</v>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Wilmington NC</t>
+        </is>
+      </c>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L114" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Drain Team Albany</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>drainteamalbany.com</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>https://www.drainteamalbany.com/</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>Dave Dingley</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>info@trinity.plumbing</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>(518) 348-3032</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>Albany NY</t>
+        </is>
+      </c>
+      <c r="I115" t="n">
+        <v>90</v>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>drain cleaning service Albany NY</t>
+        </is>
+      </c>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L115" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>ARC Plumbing</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>arcplumbing.com</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>https://arcplumbing.com/24-hour-plumber-raleigh-nc/</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>Emergency Service</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>customercare@arc.plumbing</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>919-888-3500</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>Raleigh NC</t>
+        </is>
+      </c>
+      <c r="I116" t="n">
+        <v>90</v>
+      </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>emergency plumber Raleigh NC</t>
+        </is>
+      </c>
+      <c r="K116" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L116" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Metal Roof Wilmington</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>metalroofwilmington.com</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>http://www.metalroofwilmington.com/</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr"/>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>moreinfo@metalroofwilmington.com</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>866-868-1006</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>Wilmington NC</t>
+        </is>
+      </c>
+      <c r="I117" t="n">
+        <v>84</v>
+      </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Wilmington NC</t>
+        </is>
+      </c>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L117" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-18 19:17 UTC (cycle 15)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L117"/>
+  <dimension ref="A1:L119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7260,7 +7260,6 @@
           <t>http://www.metalroofwilmington.com/</t>
         </is>
       </c>
-      <c r="E117" t="inlineStr"/>
       <c r="F117" t="inlineStr">
         <is>
           <t>moreinfo@metalroofwilmington.com</t>
@@ -7290,6 +7289,126 @@
         </is>
       </c>
       <c r="L117" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Eagle AC Heating &amp; Cooling</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>eagleacfl.com</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>https://eagleacfl.com/</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>Alex Schwartz</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>dom@imsedge.com</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>(352) 538-1533</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>Gainesville FL</t>
+        </is>
+      </c>
+      <c r="I118" t="n">
+        <v>100</v>
+      </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>heating and cooling company Gainesville FL</t>
+        </is>
+      </c>
+      <c r="K118" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L118" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Comfort Temp Heating &amp; Air</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>comforttemp.com</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>https://comforttemp.com/locations/gainesville-fl-hvac-services/</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>Share Your</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>service@comforttemp.com</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>(833) 621-5859</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>Gainesville FL</t>
+        </is>
+      </c>
+      <c r="I119" t="n">
+        <v>90</v>
+      </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>heating and cooling company Gainesville FL</t>
+        </is>
+      </c>
+      <c r="K119" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L119" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-18 19:21 UTC (cycle 18)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L119"/>
+  <dimension ref="A1:L120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7414,6 +7414,66 @@
         </is>
       </c>
     </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>wordpress-1497122-6134640.cloudwaysapps.com</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>apexelectricalac.com</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>https://apexelectricalac.com/residential-hvac-services/furnace-repair/</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>New Brau</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>info@apexelectricalac.com</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>830-407-2739</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>New Braunfels TX</t>
+        </is>
+      </c>
+      <c r="I120" t="n">
+        <v>100</v>
+      </c>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>furnace repair New Braunfels TX</t>
+        </is>
+      </c>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L120" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-18 19:24 UTC (cycle 20)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L120"/>
+  <dimension ref="A1:L122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7474,6 +7474,126 @@
         </is>
       </c>
     </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Efficient Air Conditioning &amp; Heating Repair</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>efficientheatingandairconditioning.com</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>https://efficientheatingandairconditioning.com/locations/carrollton-tx.html</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>Air Conditioni</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>dispatch@efficientheatingandairconditioning.com</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>(888) 691-4668</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>Carrollton TX</t>
+        </is>
+      </c>
+      <c r="I121" t="n">
+        <v>90</v>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>air conditioning repair Carrollton TX</t>
+        </is>
+      </c>
+      <c r="K121" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L121" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>Bridges Air</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>bridgesair.com</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>https://bridgesair.com/service-area/carrollton/</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>Fort Worth</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>acservices@bridgesair.com</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>(972) 600-8511</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>Carrollton TX</t>
+        </is>
+      </c>
+      <c r="I122" t="n">
+        <v>88</v>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>air conditioning repair Carrollton TX</t>
+        </is>
+      </c>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L122" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-18 19:26 UTC (cycle 21)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L122"/>
+  <dimension ref="A1:L124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7594,6 +7594,122 @@
         </is>
       </c>
     </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>Metal Roofing | Peak Construction Roofing | Duluth, MN, Virginia, MN, Hayward, W</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>peakconstructionroofing.com</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>https://www.peakconstructionroofing.com/metal-roofing</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>Common Questions</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>office.peakroofing@gmail.com</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>(218) 728-8033</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>Duluth MN</t>
+        </is>
+      </c>
+      <c r="I123" t="n">
+        <v>100</v>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Duluth MN</t>
+        </is>
+      </c>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L123" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>My Roofing Tech</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>myroofing.tech</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>https://www.myroofing.tech/contractors/iron-ridge-construction-metal-roofing-duluth</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr"/>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>info@myroofing.tech</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>(218) 393-8735</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>Duluth MN</t>
+        </is>
+      </c>
+      <c r="I124" t="n">
+        <v>100</v>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Duluth MN</t>
+        </is>
+      </c>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L124" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-18 19:36 UTC (cycle 28)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L124"/>
+  <dimension ref="A1:L125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7675,7 +7675,6 @@
           <t>https://www.myroofing.tech/contractors/iron-ridge-construction-metal-roofing-duluth</t>
         </is>
       </c>
-      <c r="E124" t="inlineStr"/>
       <c r="F124" t="inlineStr">
         <is>
           <t>info@myroofing.tech</t>
@@ -7705,6 +7704,66 @@
         </is>
       </c>
       <c r="L124" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>Frisco TX Water Heater</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>friscowaterheater.com</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>https://friscowaterheater.com/</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>Water Heater</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>service@friscowaterheater.com</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>972-843-1316</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>Frisco TX</t>
+        </is>
+      </c>
+      <c r="I125" t="n">
+        <v>94</v>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>water heater repair Frisco TX</t>
+        </is>
+      </c>
+      <c r="K125" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L125" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-18 19:38 UTC (cycle 29)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L125"/>
+  <dimension ref="A1:L127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7769,6 +7769,126 @@
         </is>
       </c>
     </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>Ideal Services</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>idealdallas.com</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>https://www.idealdallas.com/heating-furnace-repair/</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>Signs Your</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>service@idealservices.com</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>(817) 380-9631</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>Dallas TX</t>
+        </is>
+      </c>
+      <c r="I126" t="n">
+        <v>100</v>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>furnace repair Dallas TX</t>
+        </is>
+      </c>
+      <c r="K126" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L126" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>Wonder Roofing &amp; Renovations</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>wonderroofing.com</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>https://wonderroofing.com/</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>Indian River</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>info@wonderroofing.com</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>321-802-9100</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>Palm Bay FL</t>
+        </is>
+      </c>
+      <c r="I127" t="n">
+        <v>100</v>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>roofer Palm Bay FL</t>
+        </is>
+      </c>
+      <c r="K127" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L127" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-18 19:51 UTC (cycle 38)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L127"/>
+  <dimension ref="A1:L128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7889,6 +7889,62 @@
         </is>
       </c>
     </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>Tempo Air</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>tempoair.com</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>https://tempoair.com/locations/ac-service-irving/</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr"/>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>info@tempoair.com</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>972-579-2000</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>Irving TX</t>
+        </is>
+      </c>
+      <c r="I128" t="n">
+        <v>90</v>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>air conditioning repair Irving TX</t>
+        </is>
+      </c>
+      <c r="K128" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L128" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-18 19:57 UTC (cycle 42)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L128"/>
+  <dimension ref="A1:L131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7910,7 +7910,6 @@
           <t>https://tempoair.com/locations/ac-service-irving/</t>
         </is>
       </c>
-      <c r="E128" t="inlineStr"/>
       <c r="F128" t="inlineStr">
         <is>
           <t>info@tempoair.com</t>
@@ -7940,6 +7939,178 @@
         </is>
       </c>
       <c r="L128" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>Budd Mechanical Systems</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>buddmechanical.com</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>https://buddmechanical.com/citystate/hammond-in/</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>See What</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>dbooth@buddmechanical.com</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>219-931-1073</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>Hammond IN</t>
+        </is>
+      </c>
+      <c r="I129" t="n">
+        <v>100</v>
+      </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>furnace repair Hammond IN</t>
+        </is>
+      </c>
+      <c r="K129" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L129" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>Roofer Fort Lauderdale</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>drrooferfortlauderdale.com</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>https://drrooferfortlauderdale.com/</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr"/>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>cs@drrooferflorida.com</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>(954) 210-4374</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>Fort Lauderdale FL</t>
+        </is>
+      </c>
+      <c r="I130" t="n">
+        <v>90</v>
+      </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>roofer Fort Lauderdale FL</t>
+        </is>
+      </c>
+      <c r="K130" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L130" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>Fort Lauderdale Roofing</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>fortlauderdaleroofing.com</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>http://fortlauderdaleroofing.com/</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr"/>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>info@fortlauderdaleroofing.com</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>(954) 903-1656</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>Fort Lauderdale FL</t>
+        </is>
+      </c>
+      <c r="I131" t="n">
+        <v>66</v>
+      </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>roofer Fort Lauderdale FL</t>
+        </is>
+      </c>
+      <c r="K131" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L131" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-18 19:58 UTC (cycle 43)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L131"/>
+  <dimension ref="A1:L132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8025,7 +8025,6 @@
           <t>https://drrooferfortlauderdale.com/</t>
         </is>
       </c>
-      <c r="E130" t="inlineStr"/>
       <c r="F130" t="inlineStr">
         <is>
           <t>cs@drrooferflorida.com</t>
@@ -8081,7 +8080,6 @@
           <t>http://fortlauderdaleroofing.com/</t>
         </is>
       </c>
-      <c r="E131" t="inlineStr"/>
       <c r="F131" t="inlineStr">
         <is>
           <t>info@fortlauderdaleroofing.com</t>
@@ -8111,6 +8109,66 @@
         </is>
       </c>
       <c r="L131" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>S &amp; B Plumbing</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>sbplumbingutah.com</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>https://www.sbplumbingutah.com/</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>Josh Harkleroad</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>sbputah@gmail.com</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>801-528-4999</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>Ogden UT</t>
+        </is>
+      </c>
+      <c r="I132" t="n">
+        <v>100</v>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>plumbing company Ogden UT</t>
+        </is>
+      </c>
+      <c r="K132" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L132" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-18 20:17 UTC (cycle 56)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L132"/>
+  <dimension ref="A1:L133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8174,6 +8174,66 @@
         </is>
       </c>
     </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>Tekton Home Solutions</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>tektonhomesolutions.com</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>https://www.tektonhomesolutions.com/mcallen/roofing/</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>Free Estimate</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>info@tektonhomesolutions.com</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>(956) 862-7643</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>McAllen TX</t>
+        </is>
+      </c>
+      <c r="I133" t="n">
+        <v>100</v>
+      </c>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>residential roofing company McAllen TX</t>
+        </is>
+      </c>
+      <c r="K133" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L133" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-18 20:24 UTC (cycle 61)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L133"/>
+  <dimension ref="A1:L135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8234,6 +8234,122 @@
         </is>
       </c>
     </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>Sullivan and Fortner Roofing Inc</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>roofingsince1910.com</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>https://www.roofingsince1910.com/services-seperator/roof-replacement</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>Miguel Gomez</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>info@sullivanfortner-roofs.com</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>(765) 447-3155</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>Lafayette IN</t>
+        </is>
+      </c>
+      <c r="I134" t="n">
+        <v>100</v>
+      </c>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>roof replacement Lafayette IN</t>
+        </is>
+      </c>
+      <c r="K134" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L134" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>On Call Heating and Air Conditiong Services in Bakersfield</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>oncallheatandair.com</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>https://oncallheatandair.com/</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr"/>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>oncallhvac@icloud.com</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>(661) 619-6887</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>Bakersfield CA</t>
+        </is>
+      </c>
+      <c r="I135" t="n">
+        <v>88</v>
+      </c>
+      <c r="J135" t="inlineStr">
+        <is>
+          <t>heating and cooling company Bakersfield CA</t>
+        </is>
+      </c>
+      <c r="K135" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L135" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-18 20:27 UTC (cycle 63)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L135"/>
+  <dimension ref="A1:L136"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8315,7 +8315,6 @@
           <t>https://oncallheatandair.com/</t>
         </is>
       </c>
-      <c r="E135" t="inlineStr"/>
       <c r="F135" t="inlineStr">
         <is>
           <t>oncallhvac@icloud.com</t>
@@ -8345,6 +8344,66 @@
         </is>
       </c>
       <c r="L135" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>Sewer Line Repair in Kissimmee, FL | Same-Day Service</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>goodplumbersfl.com</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>https://goodplumbersfl.com/kissimmee-fl/sewer-line-repair</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>Michael Cole</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>info@goodplumbersfl.com</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>(786) 675-4030</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>Kissimmee FL</t>
+        </is>
+      </c>
+      <c r="I136" t="n">
+        <v>90</v>
+      </c>
+      <c r="J136" t="inlineStr">
+        <is>
+          <t>sewer repair Kissimmee FL</t>
+        </is>
+      </c>
+      <c r="K136" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L136" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-18 20:39 UTC (cycle 71)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L136"/>
+  <dimension ref="A1:L137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8409,6 +8409,62 @@
         </is>
       </c>
     </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>FLOW GO</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>flowgosolutions.com</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>https://www.flowgosolutions.com/</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr"/>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>services@flowgosolutions.com</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>(843) 653-6353</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>Charleston SC</t>
+        </is>
+      </c>
+      <c r="I137" t="n">
+        <v>88</v>
+      </c>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t>drain cleaning service Charleston SC</t>
+        </is>
+      </c>
+      <c r="K137" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L137" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-18 21:04 UTC (cycle 88)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L137"/>
+  <dimension ref="A1:L139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8430,7 +8430,6 @@
           <t>https://www.flowgosolutions.com/</t>
         </is>
       </c>
-      <c r="E137" t="inlineStr"/>
       <c r="F137" t="inlineStr">
         <is>
           <t>services@flowgosolutions.com</t>
@@ -8460,6 +8459,122 @@
         </is>
       </c>
       <c r="L137" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>Roofers | Wichita, KS | Wichita Roof Consultants</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>wichitaroofconsultants.com</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>https://www.wichitaroofconsultants.com/</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>Inspections We</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>wichitaroofconsultants@gmail.com</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>(316) 241-9927</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>Wichita KS</t>
+        </is>
+      </c>
+      <c r="I138" t="n">
+        <v>100</v>
+      </c>
+      <c r="J138" t="inlineStr">
+        <is>
+          <t>roofer Wichita KS</t>
+        </is>
+      </c>
+      <c r="K138" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L138" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>Metal Roofing California</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>metalroofingcalifornia.com</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>https://metalroofingcalifornia.com/about/</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr"/>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>sales-mrc@metaldeck.com</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>(909) 467-2016</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>Ontario CA</t>
+        </is>
+      </c>
+      <c r="I139" t="n">
+        <v>88</v>
+      </c>
+      <c r="J139" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Ontario CA</t>
+        </is>
+      </c>
+      <c r="K139" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L139" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-18 21:05 UTC (cycle 89)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L139"/>
+  <dimension ref="A1:L140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8545,7 +8545,6 @@
           <t>https://metalroofingcalifornia.com/about/</t>
         </is>
       </c>
-      <c r="E139" t="inlineStr"/>
       <c r="F139" t="inlineStr">
         <is>
           <t>sales-mrc@metaldeck.com</t>
@@ -8575,6 +8574,62 @@
         </is>
       </c>
       <c r="L139" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>Able Island Plumbing</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>ableislandplumbing.com</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>https://ableislandplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr"/>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>info@ableislandplumbing.com</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>(718) 720-3766</t>
+        </is>
+      </c>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>Staten Island NY</t>
+        </is>
+      </c>
+      <c r="I140" t="n">
+        <v>86</v>
+      </c>
+      <c r="J140" t="inlineStr">
+        <is>
+          <t>sewer repair Staten Island NY</t>
+        </is>
+      </c>
+      <c r="K140" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L140" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-18 21:07 UTC (cycle 90)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L140"/>
+  <dimension ref="A1:L141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8600,7 +8600,6 @@
           <t>https://ableislandplumbing.com/</t>
         </is>
       </c>
-      <c r="E140" t="inlineStr"/>
       <c r="F140" t="inlineStr">
         <is>
           <t>info@ableislandplumbing.com</t>
@@ -8630,6 +8629,66 @@
         </is>
       </c>
       <c r="L140" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>Bravo Roofing</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>bravoroofingmd.com</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>https://bravoroofingmd.com/roofing-company-rockville-md/</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>Blog Seasonal</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>info@bravoroofingmd.com</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>(443) 450-6110</t>
+        </is>
+      </c>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>Rockville MD</t>
+        </is>
+      </c>
+      <c r="I141" t="n">
+        <v>100</v>
+      </c>
+      <c r="J141" t="inlineStr">
+        <is>
+          <t>roof repair company Rockville MD</t>
+        </is>
+      </c>
+      <c r="K141" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L141" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-18 21:16 UTC (cycle 96)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L141"/>
+  <dimension ref="A1:L142"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8694,6 +8694,66 @@
         </is>
       </c>
     </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>Econo Roofing</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>econo-roofing.com</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>https://econo-roofing.com/</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>Central Valley</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>econoroofing209@gmail.com</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>(209) 668-6222</t>
+        </is>
+      </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>Modesto CA</t>
+        </is>
+      </c>
+      <c r="I142" t="n">
+        <v>100</v>
+      </c>
+      <c r="J142" t="inlineStr">
+        <is>
+          <t>roofing contractor Modesto CA</t>
+        </is>
+      </c>
+      <c r="K142" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L142" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-18 21:23 UTC (cycle 101)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L142"/>
+  <dimension ref="A1:L143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8754,6 +8754,58 @@
         </is>
       </c>
     </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>Doctor Drains professional sewer and drain cleaning services in Aurora, IL and s</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>doctor-drains.com</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>https://doctor-drains.com/</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr"/>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>doctordrain.sewercleaning@gmail.com</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr"/>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>Aurora IL</t>
+        </is>
+      </c>
+      <c r="I143" t="n">
+        <v>68</v>
+      </c>
+      <c r="J143" t="inlineStr">
+        <is>
+          <t>drain cleaning service Aurora IL</t>
+        </is>
+      </c>
+      <c r="K143" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L143" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-18 21:32 UTC (cycle 107)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L143"/>
+  <dimension ref="A1:L144"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8775,13 +8775,11 @@
           <t>https://doctor-drains.com/</t>
         </is>
       </c>
-      <c r="E143" t="inlineStr"/>
       <c r="F143" t="inlineStr">
         <is>
           <t>doctordrain.sewercleaning@gmail.com</t>
         </is>
       </c>
-      <c r="G143" t="inlineStr"/>
       <c r="H143" t="inlineStr">
         <is>
           <t>Aurora IL</t>
@@ -8801,6 +8799,66 @@
         </is>
       </c>
       <c r="L143" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>Sal's Heating &amp; Cooling, Plumbing &amp; Sewer</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>salslouisville.com</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>https://salslouisville.com/plumbing-services/water-heater-repair/</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>Call Us</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>salskyweb@ufhs.net</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>(502) 385-4772</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>Louisville KY</t>
+        </is>
+      </c>
+      <c r="I144" t="n">
+        <v>100</v>
+      </c>
+      <c r="J144" t="inlineStr">
+        <is>
+          <t>water heater repair Louisville KY</t>
+        </is>
+      </c>
+      <c r="K144" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L144" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-18 21:38 UTC (cycle 111)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L144"/>
+  <dimension ref="A1:L145"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8864,6 +8864,66 @@
         </is>
       </c>
     </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>Oakland Roof Repairs</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>roofrepairsoakland.com</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>https://roofrepairsoakland.com/</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>Emergency Repair</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>contact@myohanaroof.com</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>407-584-1062</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>Oakland CA</t>
+        </is>
+      </c>
+      <c r="I145" t="n">
+        <v>100</v>
+      </c>
+      <c r="J145" t="inlineStr">
+        <is>
+          <t>roof repair company Oakland CA</t>
+        </is>
+      </c>
+      <c r="K145" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L145" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-18 21:48 UTC (cycle 118)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L145"/>
+  <dimension ref="A1:L146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8924,6 +8924,66 @@
         </is>
       </c>
     </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>Winston-Salem, NC Furnace Repair</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>gwynservices.com</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>https://www.gwynservices.com/winston-salem/furnace-repair</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>Gwyn Owner</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>contact@gwynservices.com</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>336-774-1818</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>Winston Salem NC</t>
+        </is>
+      </c>
+      <c r="I146" t="n">
+        <v>90</v>
+      </c>
+      <c r="J146" t="inlineStr">
+        <is>
+          <t>furnace repair Winston Salem NC</t>
+        </is>
+      </c>
+      <c r="K146" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L146" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-18 21:51 UTC (cycle 120)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L146"/>
+  <dimension ref="A1:L147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8984,6 +8984,66 @@
         </is>
       </c>
     </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>Roof Angels Metal Roof Repair — Amarillo, TX</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>amarillo-tx.roofangels.org</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>https://amarillo-tx.roofangels.org/services/metal-roof-repair/</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>Experience Metal</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>info@roofangels.org</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>(877) 510-0035</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>Amarillo TX</t>
+        </is>
+      </c>
+      <c r="I147" t="n">
+        <v>90</v>
+      </c>
+      <c r="J147" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Amarillo TX</t>
+        </is>
+      </c>
+      <c r="K147" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L147" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-18 21:55 UTC (cycle 123)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L147"/>
+  <dimension ref="A1:L148"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9044,6 +9044,66 @@
         </is>
       </c>
     </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>alschmidtroofing.com</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>alschmidtroofing.com</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>https://alschmidtroofing.com/</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>Inspection Serving</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>saksham@a8c.in</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>(352) 652-8462</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>Gainesville FL</t>
+        </is>
+      </c>
+      <c r="I148" t="n">
+        <v>100</v>
+      </c>
+      <c r="J148" t="inlineStr">
+        <is>
+          <t>roof repair company Gainesville FL</t>
+        </is>
+      </c>
+      <c r="K148" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L148" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-18 21:59 UTC (cycle 126)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L148"/>
+  <dimension ref="A1:L150"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9104,6 +9104,122 @@
         </is>
       </c>
     </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>Plumbing Services | Cooper Plumbing Repair and Maintenance | Baton Rouge, LA</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>cooperplumbing.org</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>https://www.cooperplumbing.org/</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>Saint Francisville</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>shaun.f.cooper1985@gmail.com</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>(225) 241-9289</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>Baton Rouge LA</t>
+        </is>
+      </c>
+      <c r="I149" t="n">
+        <v>100</v>
+      </c>
+      <c r="J149" t="inlineStr">
+        <is>
+          <t>plumbing company Baton Rouge LA</t>
+        </is>
+      </c>
+      <c r="K149" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L149" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>Trinity Plumbing</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>trinityplumbingla.com</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>https://www.trinityplumbingla.com/</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr"/>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>inbox@trinityplumbingla.com</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>225-501-5554</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>Baton Rouge LA</t>
+        </is>
+      </c>
+      <c r="I150" t="n">
+        <v>100</v>
+      </c>
+      <c r="J150" t="inlineStr">
+        <is>
+          <t>plumbing company Baton Rouge LA</t>
+        </is>
+      </c>
+      <c r="K150" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L150" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-18 22:05 UTC (cycle 130)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L150"/>
+  <dimension ref="A1:L151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9185,7 +9185,6 @@
           <t>https://www.trinityplumbingla.com/</t>
         </is>
       </c>
-      <c r="E150" t="inlineStr"/>
       <c r="F150" t="inlineStr">
         <is>
           <t>inbox@trinityplumbingla.com</t>
@@ -9215,6 +9214,62 @@
         </is>
       </c>
       <c r="L150" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>Hubbell</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>hubbellmech.com</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>https://hubbellmech.com/heat-pump-systems-dealer-installer-santa-fe/</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr"/>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>onstadjohn@gmail.com</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>505-471-4221</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>Santa Fe NM</t>
+        </is>
+      </c>
+      <c r="I151" t="n">
+        <v>90</v>
+      </c>
+      <c r="J151" t="inlineStr">
+        <is>
+          <t>heat pump installation Santa Fe NM</t>
+        </is>
+      </c>
+      <c r="K151" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L151" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-18 22:33 UTC (cycle 149)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L151"/>
+  <dimension ref="A1:L152"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9240,7 +9240,6 @@
           <t>https://hubbellmech.com/heat-pump-systems-dealer-installer-santa-fe/</t>
         </is>
       </c>
-      <c r="E151" t="inlineStr"/>
       <c r="F151" t="inlineStr">
         <is>
           <t>onstadjohn@gmail.com</t>
@@ -9270,6 +9269,66 @@
         </is>
       </c>
       <c r="L151" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>Taylor Made Services Roofing</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>taylor-made-services.com</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>https://taylor-made-services.com/roofing-contractors-in-biloxi-ms/</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>Estimate Call</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>corporate.tmsr@gmail.com</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>251-270-1553</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>Biloxi MS</t>
+        </is>
+      </c>
+      <c r="I152" t="n">
+        <v>96</v>
+      </c>
+      <c r="J152" t="inlineStr">
+        <is>
+          <t>roofing contractor Biloxi MS</t>
+        </is>
+      </c>
+      <c r="K152" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L152" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-18 22:39 UTC (cycle 153)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L152"/>
+  <dimension ref="A1:L153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9334,6 +9334,62 @@
         </is>
       </c>
     </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>Fredericksburg Air Conditioning Repairs &amp; HVAC Heating &amp; Services: Serving Frede</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>fredericksburgheatingandcooling.com</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>https://www.fredericksburgheatingandcooling.com/</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr"/>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>fhvac@cox.net</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>540-374-1087</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>Fredericksburg VA</t>
+        </is>
+      </c>
+      <c r="I153" t="n">
+        <v>80</v>
+      </c>
+      <c r="J153" t="inlineStr">
+        <is>
+          <t>heating and cooling company Fredericksburg VA</t>
+        </is>
+      </c>
+      <c r="K153" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L153" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-18 22:42 UTC (cycle 155)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L153"/>
+  <dimension ref="A1:L154"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9355,7 +9355,6 @@
           <t>https://www.fredericksburgheatingandcooling.com/</t>
         </is>
       </c>
-      <c r="E153" t="inlineStr"/>
       <c r="F153" t="inlineStr">
         <is>
           <t>fhvac@cox.net</t>
@@ -9385,6 +9384,66 @@
         </is>
       </c>
       <c r="L153" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>Roof Repair in Syracuse, NY | EJS Contractors CNY</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>ejscontractors.com</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>https://ejscontractors.com/roof-repair</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>Years Experience</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>info@ejscontractorscny.com</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>(315) 243-4076</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>Syracuse NY</t>
+        </is>
+      </c>
+      <c r="I154" t="n">
+        <v>90</v>
+      </c>
+      <c r="J154" t="inlineStr">
+        <is>
+          <t>roof repair company Syracuse NY</t>
+        </is>
+      </c>
+      <c r="K154" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L154" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-18 22:56 UTC (cycle 165)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L154"/>
+  <dimension ref="A1:L155"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9449,6 +9449,66 @@
         </is>
       </c>
     </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>Bay Area HVAC Service</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>bayareahvacservice.com</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>https://bayareahvacservice.com/services/furnace-repair/sunnyvale/</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>San Ramon</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>andrew@adriumservice.com</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>(925) 999-4095</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>Sunnyvale CA</t>
+        </is>
+      </c>
+      <c r="I155" t="n">
+        <v>100</v>
+      </c>
+      <c r="J155" t="inlineStr">
+        <is>
+          <t>furnace repair Sunnyvale CA</t>
+        </is>
+      </c>
+      <c r="K155" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L155" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-18 23:00 UTC (cycle 168)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-18.xlsx
+++ b/output/leads_2026-09-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L155"/>
+  <dimension ref="A1:L157"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9509,6 +9509,126 @@
         </is>
       </c>
     </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>Triple Diamond Construction</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>triplediamondok.com</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>https://triplediamondok.com/service-areas/lawton-roofer-and-contractor/</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>Ok Resources</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>info@triplediamondok.com</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>(405) 895-9972</t>
+        </is>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>Lawton OK</t>
+        </is>
+      </c>
+      <c r="I156" t="n">
+        <v>100</v>
+      </c>
+      <c r="J156" t="inlineStr">
+        <is>
+          <t>roof replacement Lawton OK</t>
+        </is>
+      </c>
+      <c r="K156" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L156" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>Hodge Roofing</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>hodgeroofing.net</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>https://hodgeroofing.net/</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>Hodge Roofing</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>info@hodgeroofing.net</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>318-946-8093</t>
+        </is>
+      </c>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>Shreveport LA</t>
+        </is>
+      </c>
+      <c r="I157" t="n">
+        <v>100</v>
+      </c>
+      <c r="J157" t="inlineStr">
+        <is>
+          <t>roofer Shreveport LA</t>
+        </is>
+      </c>
+      <c r="K157" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L157" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>